<commit_message>
feat: compare product-month revenue with optional budgets
</commit_message>
<xml_diff>
--- a/public/product-template.xlsx
+++ b/public/product-template.xlsx
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t>Product Cost</t>
+  </si>
+  <si>
+    <t>Revenue Budget</t>
   </si>
   <si>
     <t>2026-01</t>
@@ -108,13 +111,16 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>120</v>
@@ -125,13 +131,16 @@
       <c r="E2">
         <v>72000</v>
       </c>
+      <c r="F2">
+        <v>110000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>60</v>
@@ -142,13 +151,16 @@
       <c r="E3">
         <v>75000</v>
       </c>
+      <c r="F3">
+        <v>160000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>140</v>
@@ -159,13 +171,16 @@
       <c r="E4">
         <v>84000</v>
       </c>
+      <c r="F4">
+        <v>150000</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
       </c>
       <c r="C5">
         <v>70</v>
@@ -176,13 +191,16 @@
       <c r="E5">
         <v>87500</v>
       </c>
+      <c r="F5">
+        <v>170000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>20</v>
@@ -193,13 +211,16 @@
       <c r="E6">
         <v>15000</v>
       </c>
+      <c r="F6">
+        <v>12000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -209,6 +230,9 @@
       </c>
       <c r="E7">
         <v>2500</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add product sales price volume and cost variances
</commit_message>
<xml_diff>
--- a/public/product-template.xlsx
+++ b/public/product-template.xlsx
@@ -32,6 +32,15 @@
   </si>
   <si>
     <t>Revenue Budget</t>
+  </si>
+  <si>
+    <t>Budgeted Units</t>
+  </si>
+  <si>
+    <t>Budgeted Selling Price</t>
+  </si>
+  <si>
+    <t>Cost Budget</t>
   </si>
   <si>
     <t>2026-01</t>
@@ -114,13 +123,22 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>120</v>
@@ -134,13 +152,22 @@
       <c r="F2">
         <v>110000</v>
       </c>
+      <c r="G2">
+        <v>100</v>
+      </c>
+      <c r="H2">
+        <v>1100</v>
+      </c>
+      <c r="I2">
+        <v>70000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>60</v>
@@ -154,13 +181,22 @@
       <c r="F3">
         <v>160000</v>
       </c>
+      <c r="G3">
+        <v>80</v>
+      </c>
+      <c r="H3">
+        <v>2000</v>
+      </c>
+      <c r="I3">
+        <v>80000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>140</v>
@@ -174,13 +210,22 @@
       <c r="F4">
         <v>150000</v>
       </c>
+      <c r="G4">
+        <v>150</v>
+      </c>
+      <c r="H4">
+        <v>1000</v>
+      </c>
+      <c r="I4">
+        <v>90000</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>70</v>
@@ -194,13 +239,22 @@
       <c r="F5">
         <v>170000</v>
       </c>
+      <c r="G5">
+        <v>68</v>
+      </c>
+      <c r="H5">
+        <v>2500</v>
+      </c>
+      <c r="I5">
+        <v>90000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>20</v>
@@ -214,13 +268,22 @@
       <c r="F6">
         <v>12000</v>
       </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>500</v>
+      </c>
+      <c r="I6">
+        <v>14000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -233,6 +296,15 @@
       </c>
       <c r="F7">
         <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>